<commit_message>
Updated all reg_*.xlsx estimates -additionally updated time_series_factor.xlsx and scenario_parametricMatching.xlsx
</commit_message>
<xml_diff>
--- a/input/ES/reg_RMSE.xlsx
+++ b/input/ES/reg_RMSE.xlsx
@@ -93,7 +93,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>0.78482760577743338</v>
+        <v>0.78446471560410957</v>
       </c>
     </row>
     <row r="3">
@@ -101,7 +101,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>0.81220364204212658</v>
+        <v>0.81018860135585247</v>
       </c>
     </row>
     <row r="4">
@@ -109,7 +109,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>0.29965633365783223</v>
+        <v>0.29717822576161473</v>
       </c>
     </row>
     <row r="5">
@@ -117,7 +117,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>0.28215882296686756</v>
+        <v>0.28159289135004328</v>
       </c>
     </row>
     <row r="6">
@@ -125,7 +125,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>1.368326066957045</v>
+        <v>1.3682056319306308</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Latest updated ES regression estimates applied
- 'Person.java': add the five shortened names the new ES estimates use as aliases of existing regressors: InvMillsRatio, Lesdf_c4_BothNotEmp_L1, Lesdf_c4_EmpSpouseNotEmp_L1, Lesdf_c4_NotEmpSpouseEmp_L1 and Reached_Retirement_Age_Les_L1. The original names still work.

- Wages and employment selection (W1*, W1*-sel): re-estimated with work history in years (Liwwh) as a new regressor; the wage RMSEs and the parametric-matching parameters are updated to match.

- U2 and R1b now use the shortened regressor names.
</commit_message>
<xml_diff>
--- a/input/ES/reg_RMSE.xlsx
+++ b/input/ES/reg_RMSE.xlsx
@@ -15,7 +15,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="7" uniqueCount="7">
   <si>
-    <t>REGRESSOR</t>
+    <t>PROCESS</t>
   </si>
   <si>
     <t>W1fa</t>
@@ -33,7 +33,7 @@
     <t>I3</t>
   </si>
   <si>
-    <t>COEFFICIENT</t>
+    <t>RMSE</t>
   </si>
 </sst>
 </file>
@@ -93,7 +93,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>0.78446471560410957</v>
+        <v>0.78675384317038055</v>
       </c>
     </row>
     <row r="3">
@@ -101,7 +101,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>0.81018860135585247</v>
+        <v>0.81075347300684897</v>
       </c>
     </row>
     <row r="4">
@@ -109,7 +109,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>0.29717822576161473</v>
+        <v>0.29712044451237502</v>
       </c>
     </row>
     <row r="5">
@@ -117,7 +117,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>0.28159289135004328</v>
+        <v>0.28158346966871511</v>
       </c>
     </row>
     <row r="6">

</xml_diff>